<commit_message>
Audit model history: best run first
The run after the speed work now leads the table. The saved run names carry
the order the runs were made in, so those numbers are dropped from the audit
rather than renumbered; the record itself (results/assistant_model_trials.csv)
is unchanged.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/results/assistant_audit.xlsx
+++ b/results/assistant_audit.xlsx
@@ -673,7 +673,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Earlier runs that chose DeepSeek: before and after the speed work, and two local models.</t>
+          <t>Earlier runs that chose DeepSeek: after and before the speed work, and two local models. Listed best first; the order the runs were made in is in results/assistant_model_trials.csv.</t>
         </is>
       </c>
     </row>
@@ -11511,7 +11511,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>1. DeepSeek, full profile, before the speed work</t>
+          <t>DeepSeek, full profile, after the speed work</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -11536,22 +11536,22 @@
         <v>18</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>14.5</v>
+        <v>5.9</v>
       </c>
       <c r="H2" s="3" t="n">
-        <v>6.2</v>
+        <v>4.8</v>
       </c>
       <c r="I2" s="3" t="n">
-        <v>145.4</v>
+        <v>13</v>
       </c>
       <c r="J2" s="3" t="n">
-        <v>0.179</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>2. DeepSeek, full profile, after the speed work</t>
+          <t>DeepSeek, full profile, before the speed work</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -11576,22 +11576,22 @@
         <v>18</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>5.9</v>
+        <v>14.5</v>
       </c>
       <c r="H3" s="3" t="n">
-        <v>4.8</v>
+        <v>6.2</v>
       </c>
       <c r="I3" s="3" t="n">
-        <v>13</v>
+        <v>145.4</v>
       </c>
       <c r="J3" s="3" t="n">
-        <v>0.1</v>
+        <v>0.179</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>3. DeepSeek, compact profile (control)</t>
+          <t>DeepSeek, compact profile (control)</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -11631,7 +11631,7 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>4. Gemma 4 26B, local, compact profile</t>
+          <t>Gemma 4 26B, local, compact profile</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -11671,7 +11671,7 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>5. Qwen3 14B, local, compact profile</t>
+          <t>Qwen3 14B, local, compact profile</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">

</xml_diff>